<commit_message>
Cross-check resolved-issue count against the shared Google Sheet (2026-09-21)
Downloaded the shared Google Sheet directly and compared its Status
column against a fresh live-site check for every row where the two
disagreed, rather than trusting either source. Confirmed 18 of the
sheet's "Done" claims are genuinely fixed as of today (5 shortcode
legacy pages now redirect, 3 ad-landing pages now noindexed, 2 pages
now 404, a slug typo fixed, a duplicate post redirects, the about-us
founding story is present, and AS-253 resolves as a side effect of
the AS-197 redirect). 23 of the sheet's "Done" claims did not hold
up: 22 portfolio project pages are still thin with no alt text
despite being marked Done, plus the known AS-037 regression.

Net: 100 of 253 tracked issues confirmed resolved as of today.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TbLUcNPxRUqBBBz7fDi7SJ
</commit_message>
<xml_diff>
--- a/seo-geo/tracking/issue-tracker-for-gsheet-import.xlsx
+++ b/seo-geo/tracking/issue-tracker-for-gsheet-import.xlsx
@@ -3942,7 +3942,11 @@
           <t>R3</t>
         </is>
       </c>
-      <c r="K63" s="2" t="inlineStr"/>
+      <c r="K63" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: live title tag now reads "Marketing division - Albert Scott" (correct spelling) and the AIOSEO breadcrumb schema no longer says "Devision". https://www.albertscott.com/marketing-division/ is now the canonical 200 page; https://www.albertscott.com/marketing-devision/ 301s to it. Note: one sitewide nav menu link still points at the old /marketing-devision/ URL, which still works via the redirect but adds an unnecessary hop; minor, not blocking this row.)</t>
+        </is>
+      </c>
       <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="2" t="inlineStr"/>
     </row>
@@ -9645,7 +9649,11 @@
           <t>R13</t>
         </is>
       </c>
-      <c r="K170" s="2" t="inlineStr"/>
+      <c r="K170" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/project/national-public-seatinf/ now 301s to the corrected slug https://www.albertscott.com/project/national-public-seating/.)</t>
+        </is>
+      </c>
       <c r="L170" s="2" t="inlineStr"/>
       <c r="M170" s="2" t="inlineStr"/>
     </row>
@@ -10334,7 +10342,11 @@
           <t>R13</t>
         </is>
       </c>
-      <c r="K183" s="2" t="inlineStr"/>
+      <c r="K183" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: same fix as AS-168, confirmed by direct request, 301 to the corrected slug.)</t>
+        </is>
+      </c>
       <c r="L183" s="2" t="inlineStr"/>
       <c r="M183" s="2" t="inlineStr"/>
     </row>
@@ -10387,7 +10399,11 @@
           <t>R12</t>
         </is>
       </c>
-      <c r="K184" s="2" t="inlineStr"/>
+      <c r="K184" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/blog/mouthwatchers/ now 301s to https://www.albertscott.com/case-studies/mouthwatchers/, exactly the recommended fix.)</t>
+        </is>
+      </c>
       <c r="L184" s="2" t="inlineStr"/>
       <c r="M184" s="2" t="inlineStr"/>
     </row>
@@ -10811,7 +10827,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K192" s="2" t="inlineStr"/>
+      <c r="K192" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/home/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L192" s="2" t="inlineStr"/>
       <c r="M192" s="2" t="inlineStr"/>
     </row>
@@ -10864,7 +10884,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K193" s="2" t="inlineStr"/>
+      <c r="K193" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/amazon-management-agency/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L193" s="2" t="inlineStr"/>
       <c r="M193" s="2" t="inlineStr"/>
     </row>
@@ -10917,7 +10941,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K194" s="2" t="inlineStr"/>
+      <c r="K194" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/for-amazon-brands/ now carries meta robots "noindex, nofollow...". Page still returns 200 but is out of the index, matching the recommended fix for an active ad landing page.)</t>
+        </is>
+      </c>
       <c r="L194" s="2" t="inlineStr"/>
       <c r="M194" s="2" t="inlineStr"/>
     </row>
@@ -10970,7 +10998,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K195" s="2" t="inlineStr"/>
+      <c r="K195" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/for-amazon-brandsv2/ now carries the same noindex robots tag.)</t>
+        </is>
+      </c>
       <c r="L195" s="2" t="inlineStr"/>
       <c r="M195" s="2" t="inlineStr"/>
     </row>
@@ -11023,7 +11055,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K196" s="2" t="inlineStr"/>
+      <c r="K196" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/amazon-growth-audit/ now carries the same noindex robots tag.)</t>
+        </is>
+      </c>
       <c r="L196" s="2" t="inlineStr"/>
       <c r="M196" s="2" t="inlineStr"/>
     </row>
@@ -11076,7 +11112,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K197" s="2" t="inlineStr"/>
+      <c r="K197" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/amazon-growth-audit-v2/ now returns 404, functionally the same outcome as the recommended delete/410.)</t>
+        </is>
+      </c>
       <c r="L197" s="2" t="inlineStr"/>
       <c r="M197" s="2" t="inlineStr"/>
     </row>
@@ -11129,7 +11169,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K198" s="2" t="inlineStr"/>
+      <c r="K198" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/form-ads-test/ now returns 404.)</t>
+        </is>
+      </c>
       <c r="L198" s="2" t="inlineStr"/>
       <c r="M198" s="2" t="inlineStr"/>
     </row>
@@ -11182,7 +11226,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K199" s="2" t="inlineStr"/>
+      <c r="K199" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/services/ now 301s to https://www.albertscott.com/. This also resolves AS-253, the pricing figure that was exposed in this page's broken shortcode text; that content is no longer served.)</t>
+        </is>
+      </c>
       <c r="L199" s="2" t="inlineStr"/>
       <c r="M199" s="2" t="inlineStr"/>
     </row>
@@ -11235,7 +11283,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K200" s="2" t="inlineStr"/>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/services-2/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L200" s="2" t="inlineStr"/>
       <c r="M200" s="2" t="inlineStr"/>
     </row>
@@ -11288,7 +11340,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K201" s="2" t="inlineStr"/>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/our-service/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L201" s="2" t="inlineStr"/>
       <c r="M201" s="2" t="inlineStr"/>
     </row>
@@ -11341,7 +11397,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K202" s="2" t="inlineStr"/>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/additional-services/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L202" s="2" t="inlineStr"/>
       <c r="M202" s="2" t="inlineStr"/>
     </row>
@@ -11394,7 +11454,11 @@
           <t>R1</t>
         </is>
       </c>
-      <c r="K203" s="2" t="inlineStr"/>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: https://www.albertscott.com/overview/ now 301s to https://www.albertscott.com/.)</t>
+        </is>
+      </c>
       <c r="L203" s="2" t="inlineStr"/>
       <c r="M203" s="2" t="inlineStr"/>
     </row>
@@ -14122,7 +14186,11 @@
           <t>new</t>
         </is>
       </c>
-      <c r="K251" s="2" t="inlineStr"/>
+      <c r="K251" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: /about-us/ now has a "Our Story" section reading "Albert Scott was founded in 2020 by David Greenblatt and Shlomo Greenblatt after seeing firsthand how difficult it had become for brands to succeed on Amazon...". The founding story is present, and the page grew from 648 to 721 words to hold it.)</t>
+        </is>
+      </c>
       <c r="L251" s="2" t="inlineStr"/>
       <c r="M251" s="2" t="inlineStr"/>
     </row>
@@ -14285,7 +14353,11 @@
           <t>new</t>
         </is>
       </c>
-      <c r="K254" s="2" t="inlineStr"/>
+      <c r="K254" s="2" t="inlineStr">
+        <is>
+          <t>Done (verified 2026-09-21: /services/ now 301s to the homepage instead of serving the broken shortcode page, so the "9% Commission" pricing text is no longer exposed. Resolved as a side effect of the AS-197 redirect.)</t>
+        </is>
+      </c>
       <c r="L254" s="2" t="inlineStr"/>
       <c r="M254" s="2" t="inlineStr"/>
     </row>

</xml_diff>